<commit_message>
Create ActionSelectLayout test for verifying layout and exit button
</commit_message>
<xml_diff>
--- a/Test Cases.xlsx
+++ b/Test Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endresshauser-my.sharepoint.com/personal/corbin_ferguson_endress_com/Documents/Thesis Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1627" documentId="11_AD4DB114E441178AC67DF4D41ED1D894683EDF27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{361B8735-BBF4-43CD-ABC6-232ECC75B30E}"/>
+  <xr:revisionPtr revIDLastSave="1637" documentId="11_AD4DB114E441178AC67DF4D41ED1D894683EDF27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D848577-258C-4138-9A60-41B0653B7391}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-4485" windowWidth="25440" windowHeight="15270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="53880" yWindow="-5145" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tests" sheetId="7" r:id="rId1"/>
@@ -24,7 +24,6 @@
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -67,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="194">
   <si>
     <t>Step</t>
   </si>
@@ -139,9 +138,6 @@
   </si>
   <si>
     <t>Validate File</t>
-  </si>
-  <si>
-    <t>Exit</t>
   </si>
   <si>
     <t>"New File" Button Pressed</t>
@@ -870,6 +866,18 @@
   </si>
   <si>
     <t>"Create Element" button pressed</t>
+  </si>
+  <si>
+    <t>ActionSelectLayout</t>
+  </si>
+  <si>
+    <t>Verify Buttons found</t>
+  </si>
+  <si>
+    <t>ImportElementButton, "CreateElementButton", "ModifyElementButton", "DeleteElementButton", "NewFileButton", "LoadFileButton", "ValidateFileButton", "SaveFileButton", "ExitActionSelect", "Minimize", "Maximize", "Close"</t>
+  </si>
+  <si>
+    <t>button names match list</t>
   </si>
 </sst>
 </file>
@@ -989,13 +997,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1960,10 +1968,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Corbin Ferguson" refreshedDate="46035.626586689817" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="17" xr:uid="{32ED145B-7CBC-4C3A-9787-F34239E1DCF7}">
   <cacheSource type="worksheet">
@@ -2391,45 +2395,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8512478-31DB-4352-AB46-996C676231F3}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.453125" customWidth="1"/>
+    <col min="2" max="2" width="34.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.453125" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.1796875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" t="s">
         <v>158</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C1" s="6" t="s">
-        <v>160</v>
-      </c>
       <c r="D1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G1">
         <f>COUNTIF(TestMaster[Test Status], "Not Implemented")</f>
         <v>15</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2">
         <f t="shared" ref="A2:A16" si="0">ROW()-1</f>
         <v>1</v>
@@ -2439,26 +2443,26 @@
         <v>Import Select Redundant Name</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G2">
         <f>COUNTIF(TestMaster[Test Status], "Pass")</f>
         <v>0</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I2">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -2468,26 +2472,26 @@
         <v>Element Quantity Creation</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" t="s">
         <v>164</v>
       </c>
-      <c r="D3" t="s">
-        <v>165</v>
-      </c>
       <c r="E3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G3">
         <f>COUNTIF(TestMaster[Test Status], "Fail")</f>
         <v>0</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I3">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -2497,17 +2501,17 @@
         <v>Nameless Module Creation</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G4">
         <f>COUNTIF(TestMaster[Test Status], "Not Run")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2517,13 +2521,13 @@
         <v>Redundant Element Creation</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E5" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2533,13 +2537,13 @@
         <v>No Element to Modify</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2549,13 +2553,13 @@
         <v>Completed Element Modification</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E7" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2565,13 +2569,13 @@
         <v>Modify into Redundant Element Name</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E8" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2581,13 +2585,13 @@
         <v>Delete No Element Type</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E9" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2597,13 +2601,13 @@
         <v>Delete Element Found</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E10" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2613,13 +2617,13 @@
         <v>Delete Module by Port</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E11" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2629,13 +2633,13 @@
         <v>New File Creation</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E12" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2645,13 +2649,13 @@
         <v>Save File</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E13" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2661,13 +2665,13 @@
         <v>Load File</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E14" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2677,26 +2681,26 @@
         <v>Validate File</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E15" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B16" t="str">
         <f>'File Manipulation Testing'!Y1</f>
-        <v>Exit</v>
+        <v>ActionSelectLayout</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2749,17 +2753,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B60DAC1D-2E28-4DF7-A44B-A179A310D91E}">
   <dimension ref="A1:F25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="56.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.453125" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="56.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>13</v>
       </c>
@@ -2769,7 +2773,7 @@
       <c r="E1" s="16"/>
       <c r="F1" s="17"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
@@ -2782,9 +2786,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="10" t="str">
@@ -2799,9 +2803,9 @@
         <v>Not Implemented</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
@@ -2809,7 +2813,7 @@
       <c r="E4" s="16"/>
       <c r="F4" s="17"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -2817,7 +2821,7 @@
       <c r="E5" s="16"/>
       <c r="F5" s="17"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="16" t="s">
         <v>7</v>
       </c>
@@ -2827,7 +2831,7 @@
       <c r="E6" s="16"/>
       <c r="F6" s="17"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -2847,273 +2851,273 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C8" t="s">
         <v>175</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <f>A8+1</f>
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>174</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <f>A9+1</f>
         <v>3</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <f t="shared" ref="A11:A25" si="0">A10+1</f>
         <v>4</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B24" t="s">
+        <v>112</v>
+      </c>
+      <c r="C24" t="s">
         <v>113</v>
       </c>
-      <c r="C24" t="s">
-        <v>114</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -3131,30 +3135,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0AB6AA-BAF4-4C64-96FE-66D32370F298}">
   <dimension ref="A1:R21"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="35.5703125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="35.54296875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="13" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.140625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="29.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.1796875" style="5" customWidth="1"/>
     <col min="10" max="10" width="24" style="5" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" style="13" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="29.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.5703125" style="5" customWidth="1"/>
-    <col min="16" max="16" width="23.85546875" style="5" customWidth="1"/>
-    <col min="17" max="17" width="18.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.7109375" style="5"/>
+    <col min="14" max="14" width="29.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.54296875" style="5" customWidth="1"/>
+    <col min="16" max="16" width="23.81640625" style="5" customWidth="1"/>
+    <col min="17" max="17" width="18.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.7265625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>14</v>
       </c>
@@ -3172,7 +3176,7 @@
       <c r="K1" s="16"/>
       <c r="L1" s="16"/>
       <c r="M1" s="16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N1" s="16"/>
       <c r="O1" s="16"/>
@@ -3180,7 +3184,7 @@
       <c r="Q1" s="16"/>
       <c r="R1" s="16"/>
     </row>
-    <row r="2" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
@@ -3220,9 +3224,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" t="str">
@@ -3238,7 +3242,7 @@
         <v>Not Implemented</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" t="str">
@@ -3254,7 +3258,7 @@
         <v>Not Implemented</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N3" s="16"/>
       <c r="O3" t="str">
@@ -3270,7 +3274,7 @@
         <v>Not Implemented</v>
       </c>
     </row>
-    <row r="4" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
         <v>6</v>
       </c>
@@ -3296,7 +3300,7 @@
       <c r="Q4" s="16"/>
       <c r="R4" s="16"/>
     </row>
-    <row r="5" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -3316,7 +3320,7 @@
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
     </row>
-    <row r="6" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="16" t="s">
         <v>7</v>
       </c>
@@ -3342,7 +3346,7 @@
       <c r="Q6" s="16"/>
       <c r="R6" s="16"/>
     </row>
-    <row r="7" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -3398,324 +3402,329 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G8" s="5">
         <v>1</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="M8" s="5">
         <v>1</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>125</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>126</v>
       </c>
       <c r="G9" s="5">
         <v>2</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I9" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="J9" s="4" t="s">
         <v>138</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>139</v>
       </c>
       <c r="M9" s="5">
         <v>2</v>
       </c>
       <c r="N9" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="P9" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="O9" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>3</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>127</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>128</v>
       </c>
       <c r="G10" s="5">
         <v>3</v>
       </c>
       <c r="H10" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="J10" s="4" t="s">
         <v>127</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>128</v>
       </c>
       <c r="M10" s="5">
         <v>3</v>
       </c>
       <c r="N10" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="P10" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="O10" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>4</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>131</v>
       </c>
       <c r="G11" s="5">
         <v>4</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="M11" s="5">
         <v>4</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P11" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>5</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>134</v>
-      </c>
       <c r="D12" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M12" s="5">
         <v>5</v>
       </c>
       <c r="N12" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="O12" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="O12" s="4" t="s">
-        <v>145</v>
-      </c>
       <c r="P12" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>6</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M13" s="5">
         <v>6</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O13" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="M14">
         <v>7</v>
       </c>
       <c r="N14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P14" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="M15" s="5">
         <v>8</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="M16">
         <v>9</v>
       </c>
       <c r="N16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P16" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="17" spans="13:16" ht="45" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="17" spans="13:16" ht="29" x14ac:dyDescent="0.35">
       <c r="M17">
         <v>10</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="18" spans="13:16" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="18" spans="13:16" x14ac:dyDescent="0.35">
       <c r="M18" s="5">
         <v>11</v>
       </c>
       <c r="N18" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P18" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="19" spans="13:16" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="13:16" x14ac:dyDescent="0.35">
       <c r="M19">
         <v>12</v>
       </c>
       <c r="N19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P19" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="13:16" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="13:16" x14ac:dyDescent="0.35">
       <c r="M20" s="5">
         <v>13</v>
       </c>
       <c r="N20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P20" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="21" spans="13:16" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="13:16" x14ac:dyDescent="0.35">
       <c r="M21">
         <v>14</v>
       </c>
       <c r="N21" t="s">
+        <v>112</v>
+      </c>
+      <c r="O21" t="s">
         <v>113</v>
       </c>
-      <c r="O21" t="s">
-        <v>114</v>
-      </c>
       <c r="P21" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="M1:R1"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="M3:N3"/>
@@ -3726,11 +3735,6 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A2:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3739,29 +3743,29 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31B60B4E-CDD0-4CEE-BA63-4F898D2F5023}">
   <dimension ref="A1:R25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.42578125" customWidth="1"/>
-    <col min="9" max="9" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.28515625" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.453125" customWidth="1"/>
+    <col min="9" max="9" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.26953125" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.5703125" customWidth="1"/>
-    <col min="16" max="16" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.54296875" customWidth="1"/>
+    <col min="16" max="16" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>16</v>
       </c>
@@ -3779,7 +3783,7 @@
       <c r="K1" s="16"/>
       <c r="L1" s="17"/>
       <c r="M1" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="N1" s="16"/>
       <c r="O1" s="16"/>
@@ -3787,7 +3791,7 @@
       <c r="Q1" s="16"/>
       <c r="R1" s="16"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
@@ -3822,9 +3826,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="8" t="str">
@@ -3839,7 +3843,7 @@
         <v>Not Implemented</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="8" t="str">
@@ -3854,7 +3858,7 @@
         <v>Not Implemented</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N3" s="16"/>
       <c r="O3" s="14" t="str">
@@ -3869,7 +3873,7 @@
         <v>Not Implemented</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
         <v>6</v>
       </c>
@@ -3895,7 +3899,7 @@
       <c r="Q4" s="16"/>
       <c r="R4" s="16"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -3915,7 +3919,7 @@
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="16" t="s">
         <v>7</v>
       </c>
@@ -3941,7 +3945,7 @@
       <c r="Q6" s="16"/>
       <c r="R6" s="16"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -3997,386 +4001,391 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>1</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M8">
         <v>1</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P8" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>2</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M9">
         <v>2</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="G10">
         <v>3</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M10">
         <v>3</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G11">
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M11">
         <v>4</v>
       </c>
       <c r="N11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O11" t="s">
+        <v>89</v>
+      </c>
+      <c r="P11" t="s">
         <v>90</v>
       </c>
-      <c r="P11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G12">
         <v>5</v>
       </c>
       <c r="H12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M12">
         <v>5</v>
       </c>
       <c r="N12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P12" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G13">
         <v>6</v>
       </c>
       <c r="H13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M13">
         <v>6</v>
       </c>
       <c r="N13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P13" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G14">
         <v>7</v>
       </c>
       <c r="H14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M14">
         <v>8</v>
       </c>
       <c r="N14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O14" t="s">
+        <v>89</v>
+      </c>
+      <c r="P14" t="s">
         <v>90</v>
       </c>
-      <c r="P14" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G15">
         <v>8</v>
       </c>
       <c r="H15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M15">
         <v>9</v>
       </c>
       <c r="N15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P15" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G16">
         <v>9</v>
       </c>
       <c r="H16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M16">
         <v>10</v>
       </c>
       <c r="N16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P16" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="17" spans="7:10" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G17">
         <v>10</v>
       </c>
       <c r="H17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J17" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G18">
         <v>11</v>
       </c>
       <c r="H18" t="s">
+        <v>101</v>
+      </c>
+      <c r="I18" t="s">
         <v>102</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>103</v>
       </c>
-      <c r="J18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G19">
         <v>12</v>
       </c>
       <c r="H19" t="s">
+        <v>88</v>
+      </c>
+      <c r="I19" t="s">
         <v>89</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>90</v>
       </c>
-      <c r="J19" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" spans="7:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G20">
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J20" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="21" spans="7:10" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G21">
         <v>14</v>
       </c>
       <c r="H21" t="s">
+        <v>106</v>
+      </c>
+      <c r="I21" t="s">
+        <v>108</v>
+      </c>
+      <c r="J21" t="s">
         <v>107</v>
       </c>
-      <c r="I21" t="s">
-        <v>109</v>
-      </c>
-      <c r="J21" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" spans="7:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G22">
         <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J22" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="23" spans="7:10" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G23">
         <v>16</v>
       </c>
       <c r="H23" t="s">
+        <v>106</v>
+      </c>
+      <c r="I23" t="s">
+        <v>108</v>
+      </c>
+      <c r="J23" t="s">
         <v>107</v>
       </c>
-      <c r="I23" t="s">
-        <v>109</v>
-      </c>
-      <c r="J23" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="24" spans="7:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G24">
         <v>17</v>
       </c>
       <c r="H24" t="s">
+        <v>112</v>
+      </c>
+      <c r="I24" t="s">
         <v>113</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>114</v>
       </c>
-      <c r="J24" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="25" spans="7:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="7:10" x14ac:dyDescent="0.35">
       <c r="G25">
         <v>18</v>
       </c>
       <c r="H25" t="s">
+        <v>101</v>
+      </c>
+      <c r="I25" t="s">
         <v>102</v>
       </c>
-      <c r="I25" t="s">
-        <v>103</v>
-      </c>
       <c r="J25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
     <mergeCell ref="M1:R1"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="M3:N3"/>
@@ -4387,11 +4396,6 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4400,30 +4404,29 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{791F26CA-73F7-4CFD-B892-FF534C61ED87}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.5703125" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.54296875" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.42578125" customWidth="1"/>
-    <col min="17" max="17" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.7109375"/>
+    <col min="14" max="14" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32.453125" customWidth="1"/>
+    <col min="17" max="17" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>18</v>
       </c>
@@ -4449,7 +4452,7 @@
       <c r="Q1" s="16"/>
       <c r="R1" s="16"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
@@ -4484,9 +4487,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="8" t="str">
@@ -4501,7 +4504,7 @@
         <v>Not Implemented</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="8" t="str">
@@ -4516,7 +4519,7 @@
         <v>Not Implemented</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N3" s="16"/>
       <c r="O3" s="8" t="str">
@@ -4531,55 +4534,55 @@
         <v>Not Implemented</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A4" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A6" s="16" t="s">
         <v>71</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
-        <v>72</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
@@ -4603,7 +4606,7 @@
       <c r="Q6" s="16"/>
       <c r="R6" s="16"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -4659,130 +4662,135 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:18" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>74</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="4">
         <v>1</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="4">
         <v>1</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" s="4" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9" s="15"/>
       <c r="G9" s="4">
         <v>2</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L9" s="15"/>
       <c r="M9" s="4">
         <v>2</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="F10" s="15"/>
       <c r="G10" s="4">
         <v>3</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="4">
         <v>3</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="M11" s="4">
         <v>4</v>
       </c>
       <c r="N11" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="O11" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="O11" s="4" t="s">
+      <c r="P11" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>86</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
     <mergeCell ref="M1:R1"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="M3:N3"/>
@@ -4793,11 +4801,6 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4806,40 +4809,40 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4413619-C528-4B04-A1ED-B4C77CA83066}">
   <dimension ref="A1:AD12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" style="9"/>
+    <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7265625" style="9"/>
     <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="48.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" style="9"/>
+    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="48.81640625" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" style="9"/>
     <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30.85546875" customWidth="1"/>
-    <col min="16" max="16" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.7109375" style="9"/>
+    <col min="14" max="14" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="30.81640625" customWidth="1"/>
+    <col min="16" max="16" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.7265625" style="9"/>
     <col min="19" max="19" width="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.26953125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="41" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.7109375" style="9"/>
+    <col min="22" max="22" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.7265625" style="9"/>
     <col min="25" max="25" width="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>11</v>
       </c>
@@ -4873,7 +4876,7 @@
       <c r="W1" s="16"/>
       <c r="X1" s="17"/>
       <c r="Y1" s="16" t="s">
-        <v>24</v>
+        <v>190</v>
       </c>
       <c r="Z1" s="16"/>
       <c r="AA1" s="16"/>
@@ -4881,7 +4884,7 @@
       <c r="AC1" s="16"/>
       <c r="AD1" s="16"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
@@ -4938,9 +4941,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" t="str">
@@ -4955,7 +4958,7 @@
         <v>High</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="8" t="str">
@@ -4970,7 +4973,7 @@
         <v>High</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N3" s="16"/>
       <c r="O3" s="8" t="str">
@@ -4985,7 +4988,7 @@
         <v>Medium</v>
       </c>
       <c r="S3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="T3" s="16"/>
       <c r="U3" s="8" t="str">
@@ -5000,7 +5003,7 @@
         <v>Low</v>
       </c>
       <c r="Y3" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Z3" s="16"/>
       <c r="AA3" s="8" t="str">
@@ -5015,83 +5018,83 @@
         <v>High</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="19" t="s">
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="20"/>
+      <c r="X4" s="21"/>
+      <c r="Y4" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="Z4" s="20"/>
+      <c r="AA4" s="20"/>
+      <c r="AB4" s="20"/>
+      <c r="AC4" s="20"/>
+      <c r="AD4" s="20"/>
+    </row>
+    <row r="5" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="20"/>
+      <c r="X5" s="21"/>
+      <c r="Y5" s="20"/>
+      <c r="Z5" s="20"/>
+      <c r="AA5" s="20"/>
+      <c r="AB5" s="20"/>
+      <c r="AC5" s="20"/>
+      <c r="AD5" s="20"/>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="A6" s="16" t="s">
         <v>68</v>
-      </c>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="20"/>
-      <c r="Y4" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z4" s="19"/>
-      <c r="AA4" s="19"/>
-      <c r="AB4" s="19"/>
-      <c r="AC4" s="19"/>
-      <c r="AD4" s="19"/>
-    </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="20"/>
-      <c r="Y5" s="19"/>
-      <c r="Z5" s="19"/>
-      <c r="AA5" s="19"/>
-      <c r="AB5" s="19"/>
-      <c r="AC5" s="19"/>
-      <c r="AD5" s="19"/>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
-        <v>69</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
@@ -5099,7 +5102,7 @@
       <c r="E6" s="16"/>
       <c r="F6" s="17"/>
       <c r="G6" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
@@ -5107,7 +5110,7 @@
       <c r="K6" s="16"/>
       <c r="L6" s="17"/>
       <c r="M6" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
@@ -5115,7 +5118,7 @@
       <c r="Q6" s="16"/>
       <c r="R6" s="17"/>
       <c r="S6" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="T6" s="16"/>
       <c r="U6" s="16"/>
@@ -5123,7 +5126,7 @@
       <c r="W6" s="16"/>
       <c r="X6" s="17"/>
       <c r="Y6" s="16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Z6" s="16"/>
       <c r="AA6" s="16"/>
@@ -5131,7 +5134,7 @@
       <c r="AC6" s="16"/>
       <c r="AD6" s="16"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -5223,229 +5226,231 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M8">
         <v>1</v>
       </c>
       <c r="N8" t="s">
+        <v>40</v>
+      </c>
+      <c r="O8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P8" t="s">
         <v>41</v>
-      </c>
-      <c r="O8" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" t="s">
-        <v>42</v>
       </c>
       <c r="S8">
         <v>1</v>
       </c>
       <c r="T8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="U8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Y8">
         <v>1</v>
       </c>
       <c r="Z8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AA8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AB8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" ht="58" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
       <c r="H9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M9">
         <v>2</v>
       </c>
       <c r="N9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O9" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="P9" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="S9">
         <v>2</v>
       </c>
       <c r="T9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="U9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Y9">
         <v>2</v>
       </c>
       <c r="Z9" t="s">
-        <v>64</v>
+        <v>191</v>
       </c>
       <c r="AA9" t="s">
-        <v>27</v>
+        <v>192</v>
       </c>
       <c r="AB9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G10">
         <v>3</v>
       </c>
       <c r="H10" t="s">
+        <v>49</v>
+      </c>
+      <c r="I10" t="s">
         <v>50</v>
       </c>
-      <c r="I10" t="s">
-        <v>51</v>
-      </c>
       <c r="J10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M10">
         <v>3</v>
       </c>
       <c r="N10" t="s">
+        <v>45</v>
+      </c>
+      <c r="O10" t="s">
         <v>46</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="S10">
         <v>3</v>
       </c>
       <c r="T10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U10" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+      <c r="Y10">
+        <v>3</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>4</v>
       </c>
       <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
         <v>30</v>
       </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="S11">
         <v>4</v>
       </c>
       <c r="T11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="U11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>5</v>
       </c>
       <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
         <v>32</v>
       </c>
-      <c r="C12" t="s">
-        <v>33</v>
-      </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="S12">
         <v>5</v>
       </c>
       <c r="T12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="U12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="Y1:AD1"/>
-    <mergeCell ref="Y2:Z2"/>
-    <mergeCell ref="Y3:Z3"/>
-    <mergeCell ref="S4:X5"/>
-    <mergeCell ref="S6:X6"/>
-    <mergeCell ref="Y4:AD5"/>
-    <mergeCell ref="Y6:AD6"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="S1:X1"/>
     <mergeCell ref="A4:F5"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A1:F1"/>
@@ -5461,6 +5466,16 @@
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="M3:N3"/>
+    <mergeCell ref="Y1:AD1"/>
+    <mergeCell ref="Y2:Z2"/>
+    <mergeCell ref="Y3:Z3"/>
+    <mergeCell ref="S4:X5"/>
+    <mergeCell ref="S6:X6"/>
+    <mergeCell ref="Y4:AD5"/>
+    <mergeCell ref="Y6:AD6"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="S1:X1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implement TestHelper, create FileManagementTesting up to file selection for loadFile
</commit_message>
<xml_diff>
--- a/Test Cases.xlsx
+++ b/Test Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endresshauser-my.sharepoint.com/personal/corbin_ferguson_endress_com/Documents/Thesis Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1637" documentId="11_AD4DB114E441178AC67DF4D41ED1D894683EDF27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D848577-258C-4138-9A60-41B0653B7391}"/>
+  <xr:revisionPtr revIDLastSave="1699" documentId="11_AD4DB114E441178AC67DF4D41ED1D894683EDF27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F63269EF-56D4-480B-B9BE-A1F71BFA4520}"/>
   <bookViews>
     <workbookView xWindow="53880" yWindow="-5145" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="187">
   <si>
     <t>Step</t>
   </si>
@@ -101,12 +101,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>New File Creation</t>
-  </si>
-  <si>
-    <t>Description: Test the creation of an empty template file, overwriting the existing file.</t>
-  </si>
-  <si>
     <t>Import Select Redundant Name</t>
   </si>
   <si>
@@ -131,15 +125,6 @@
     <t>Delete Module by Port</t>
   </si>
   <si>
-    <t>Save File</t>
-  </si>
-  <si>
-    <t>Load File</t>
-  </si>
-  <si>
-    <t>Validate File</t>
-  </si>
-  <si>
     <t>"New File" Button Pressed</t>
   </si>
   <si>
@@ -155,18 +140,6 @@
     <t>"ok" button Press</t>
   </si>
   <si>
-    <t>Repeat step 1</t>
-  </si>
-  <si>
-    <t>"new" button press</t>
-  </si>
-  <si>
-    <t>Cancel File Creation</t>
-  </si>
-  <si>
-    <t>"No Button Press"</t>
-  </si>
-  <si>
     <t>"Save File" Button Pressed</t>
   </si>
   <si>
@@ -197,64 +170,18 @@
     <t>File to load selected</t>
   </si>
   <si>
-    <t>C:\Users\i01505732\OneDrive - Endress+Hauser\Thesis Work\CodeProjects\L5XFiles\TemplateFiles\BasicControllertags.L5X</t>
-  </si>
-  <si>
     <t>doc object in Execute.cs updated to new object</t>
   </si>
   <si>
-    <t>Verify New File Loaded</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Check </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>one of the subobjects</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>subobject</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> exists</t>
-    </r>
-  </si>
-  <si>
     <t>Confirm File Creation</t>
   </si>
   <si>
-    <t>Verify File Saved</t>
-  </si>
-  <si>
-    <t>Check file exists at expected location</t>
-  </si>
-  <si>
     <t>"Validate" button pressed</t>
   </si>
   <si>
     <t>Preconditions: Empty template file loaded into application</t>
   </si>
   <si>
-    <t>"Ok"</t>
-  </si>
-  <si>
     <t>Load File with error</t>
   </si>
   <si>
@@ -270,9 +197,6 @@
     <t>New file created at location, return to action select window</t>
   </si>
   <si>
-    <t>File found</t>
-  </si>
-  <si>
     <t>File successfully loaded</t>
   </si>
   <si>
@@ -294,13 +218,7 @@
     <t>Launch exe</t>
   </si>
   <si>
-    <t>Description: Test the saving of a file.</t>
-  </si>
-  <si>
     <t>Preconditions: None</t>
-  </si>
-  <si>
-    <t>Preconditions: File to load.</t>
   </si>
   <si>
     <t>Description: Testing that attempting to delete an element when no element exists causes a popup</t>
@@ -859,9 +777,6 @@
     <t>Test Priority:</t>
   </si>
   <si>
-    <t>Test Priority: Low</t>
-  </si>
-  <si>
     <t>Select Quantity</t>
   </si>
   <si>
@@ -878,6 +793,45 @@
   </si>
   <si>
     <t>button names match list</t>
+  </si>
+  <si>
+    <t>Verify all buttons onscreen</t>
+  </si>
+  <si>
+    <t>buttons</t>
+  </si>
+  <si>
+    <t>no buttons found offscreen</t>
+  </si>
+  <si>
+    <t>Description: Test that the ActionSelect window launches with all necessary buttons, and that the exit button closes the window.</t>
+  </si>
+  <si>
+    <t>FileManagementTesting</t>
+  </si>
+  <si>
+    <t>"Ok" pressed</t>
+  </si>
+  <si>
+    <t>Description: Test that the file manipulation buttons are functional.</t>
+  </si>
+  <si>
+    <t>ValidateFileButton</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>LoadFileButton</t>
+  </si>
+  <si>
+    <t>.\Thesis Work\CodeProjects\L5XFiles\TestingFiles\BrokenXML.L5X</t>
+  </si>
+  <si>
+    <t>Description: Test that action select cannot be manipulated during operations.</t>
+  </si>
+  <si>
+    <t>ActionSelectLosecontrol</t>
   </si>
 </sst>
 </file>
@@ -953,13 +907,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1004,6 +957,19 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1939,7 +1905,7 @@
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>217487</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2114,8 +2080,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C34A821-A8AD-4FEE-8065-115AD927679E}" name="TestMaster" displayName="TestMaster" ref="A1:E16">
-  <autoFilter ref="A1:E16" xr:uid="{8C34A821-A8AD-4FEE-8065-115AD927679E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C34A821-A8AD-4FEE-8065-115AD927679E}" name="TestMaster" displayName="TestMaster" ref="A1:E14">
+  <autoFilter ref="A1:E14" xr:uid="{8C34A821-A8AD-4FEE-8065-115AD927679E}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{0D10C69B-6EC1-4AEC-8C25-C7145B24EE5C}" name="Test ID" totalsRowLabel="Total" dataDxfId="6">
       <calculatedColumnFormula>ROW()-1</calculatedColumnFormula>
@@ -2394,12 +2360,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8512478-31DB-4352-AB46-996C676231F3}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
     <col min="2" max="2" width="34.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1796875" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.453125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.1796875" bestFit="1" customWidth="1"/>
@@ -2408,55 +2374,55 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
       <c r="B1" t="s">
-        <v>158</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>159</v>
+        <v>139</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="D1" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="E1" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="G1">
         <f>COUNTIF(TestMaster[Test Status], "Not Implemented")</f>
-        <v>15</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>169</v>
+        <v>13</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>150</v>
       </c>
       <c r="I1" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2">
-        <f t="shared" ref="A2:A16" si="0">ROW()-1</f>
+        <f t="shared" ref="A2:A13" si="0">ROW()-1</f>
         <v>1</v>
       </c>
       <c r="B2" t="str" cm="1">
         <f t="array" ref="B2">'Element Import Testing'!A1:A1</f>
         <v>Import Select Redundant Name</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>163</v>
+      <c r="C2" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="D2" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="E2" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="G2">
         <f>COUNTIF(TestMaster[Test Status], "Pass")</f>
         <v>0</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>163</v>
+      <c r="H2" s="7" t="s">
+        <v>144</v>
       </c>
       <c r="I2">
         <v>17</v>
@@ -2471,21 +2437,21 @@
         <f t="array" ref="B3">'Element Creation Testing'!A1:A1</f>
         <v>Element Quantity Creation</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>163</v>
+      <c r="C3" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="D3" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="E3" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
       <c r="G3">
         <f>COUNTIF(TestMaster[Test Status], "Fail")</f>
         <v>0</v>
       </c>
-      <c r="H3" s="8" t="s">
-        <v>170</v>
+      <c r="H3" s="7" t="s">
+        <v>151</v>
       </c>
       <c r="I3">
         <v>17</v>
@@ -2500,11 +2466,11 @@
         <f t="array" ref="B4">'Element Creation Testing'!G1:G1</f>
         <v>Nameless Module Creation</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>163</v>
+      <c r="C4" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E4" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
       <c r="G4">
         <f>COUNTIF(TestMaster[Test Status], "Not Run")</f>
@@ -2520,11 +2486,11 @@
         <f t="array" ref="B5">'Element Creation Testing'!M1:M1</f>
         <v>Redundant Element Creation</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>163</v>
+      <c r="C5" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E5" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -2536,11 +2502,11 @@
         <f>'Element Modification Testing'!A1</f>
         <v>No Element to Modify</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>163</v>
+      <c r="C6" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E6" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -2552,11 +2518,11 @@
         <f>'Element Modification Testing'!G1</f>
         <v>Completed Element Modification</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>163</v>
+      <c r="C7" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -2568,11 +2534,11 @@
         <f>'Element Modification Testing'!M1</f>
         <v>Modify into Redundant Element Name</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>163</v>
+      <c r="C8" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E8" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -2584,11 +2550,11 @@
         <f>'Element Deletion Testing'!A1</f>
         <v>Delete No Element Type</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>163</v>
+      <c r="C9" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E9" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -2600,11 +2566,11 @@
         <f>'Element Deletion Testing'!G1</f>
         <v>Delete Element Found</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>163</v>
+      <c r="C10" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E10" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
@@ -2616,11 +2582,11 @@
         <f>'Element Deletion Testing'!M1</f>
         <v>Delete Module by Port</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>163</v>
+      <c r="C11" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E11" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -2630,13 +2596,13 @@
       </c>
       <c r="B12" t="str">
         <f>'File Manipulation Testing'!A1</f>
-        <v>New File Creation</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>163</v>
+        <v>FileManagementTesting</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E12" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -2646,61 +2612,29 @@
       </c>
       <c r="B13" t="str">
         <f>'File Manipulation Testing'!G1</f>
-        <v>Save File</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>163</v>
+        <v>ActionSelectLayout</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E13" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <f t="shared" si="0"/>
+      <c r="A14" s="21">
+        <f>ROW()-1</f>
         <v>13</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B14" s="21" t="str">
         <f>'File Manipulation Testing'!M1</f>
-        <v>Load File</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>163</v>
+        <v>ActionSelectLosecontrol</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="E14" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <f>'File Manipulation Testing'!S1</f>
-        <v>Validate File</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="E15" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <f>'File Manipulation Testing'!Y1</f>
-        <v>ActionSelectLayout</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="E16" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2719,7 +2653,7 @@
       <formula>NOT(ISERROR(SEARCH("Not Implemented",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C17:C1048576">
+  <conditionalFormatting sqref="C15:C1048576">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -2733,7 +2667,7 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{130BDE1A-E0D9-44C7-AF19-F67B1FE4D5D4}">
-      <formula1>$D$2:$D$16</formula1>
+      <formula1>$D$2:$D$14</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576" xr:uid="{0649BA16-611B-4B21-AD1C-F4AC893E68EF}">
       <formula1>"Low,Medium,High"</formula1>
@@ -2760,25 +2694,25 @@
     <col min="3" max="3" width="48.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="56.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
+      <c r="A1" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="8">
+      <c r="B2" s="15"/>
+      <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>1</v>
       </c>
@@ -2787,49 +2721,49 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="10" t="str">
+      <c r="A3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="15"/>
+      <c r="C3" s="9" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="str">
+      <c r="F3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="16" t="s">
-        <v>183</v>
-      </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
+      <c r="A4" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="16"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="16"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -2841,13 +2775,13 @@
       <c r="C7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="10" t="s">
         <v>1</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="11" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2856,268 +2790,268 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C8" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
+      <c r="A9" s="4">
         <f>A8+1</f>
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>123</v>
+      <c r="B9" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="5">
+      <c r="A10" s="4">
         <f>A9+1</f>
         <v>3</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>125</v>
+      <c r="B10" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="5">
+      <c r="A11" s="4">
         <f t="shared" ref="A11:A25" si="0">A10+1</f>
         <v>4</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>185</v>
+      <c r="B11" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="5">
+      <c r="A12" s="4">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>27</v>
+      <c r="B12" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>179</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="5">
+      <c r="A13" s="4">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>125</v>
+      <c r="B13" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="5">
+      <c r="A14" s="4">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>181</v>
+      <c r="B14" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="5">
+      <c r="A15" s="4">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="C15" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>180</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="5">
+      <c r="A16" s="4">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>27</v>
+      <c r="B16" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>179</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="5">
+      <c r="A17" s="4">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>125</v>
+      <c r="B17" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="5">
+      <c r="A18" s="4">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>127</v>
+      <c r="B18" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="5">
+      <c r="A19" s="4">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="C19" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="5">
+      <c r="A20" s="4">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>27</v>
+      <c r="B20" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>179</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="5">
+      <c r="A21" s="4">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="5">
+      <c r="A22" s="4">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>111</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>184</v>
+        <v>92</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>165</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="5">
+      <c r="A23" s="4">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="5">
+      <c r="A24" s="4">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="5">
+      <c r="A25" s="4">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>182</v>
+      <c r="B25" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>163</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -3137,135 +3071,135 @@
   <dimension ref="A1:R21"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.81640625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="35.54296875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="18.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.1796875" style="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.1796875" style="5" customWidth="1"/>
-    <col min="10" max="10" width="24" style="5" customWidth="1"/>
-    <col min="11" max="11" width="18.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.1796875" style="13" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="29.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.54296875" style="5" customWidth="1"/>
-    <col min="16" max="16" width="23.81640625" style="5" customWidth="1"/>
-    <col min="17" max="17" width="18.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.7265625" style="5"/>
+    <col min="1" max="1" width="5" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="35.54296875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="18.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.1796875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="24" style="4" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="29.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.54296875" style="4" customWidth="1"/>
+    <col min="16" max="16" width="23.81640625" style="4" customWidth="1"/>
+    <col min="17" max="17" width="18.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.7265625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
+      <c r="A1" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
     </row>
     <row r="2" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="16"/>
+      <c r="B2" s="15"/>
       <c r="C2">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>2</v>
       </c>
-      <c r="D2" s="5"/>
+      <c r="D2" s="4"/>
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="9"/>
-      <c r="G2" s="16" t="s">
+      <c r="F2" s="8"/>
+      <c r="G2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="16"/>
+      <c r="H2" s="15"/>
       <c r="I2">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>3</v>
       </c>
-      <c r="J2" s="5"/>
+      <c r="J2" s="4"/>
       <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="9"/>
-      <c r="M2" s="16" t="s">
+      <c r="L2" s="8"/>
+      <c r="M2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="16"/>
+      <c r="N2" s="15"/>
       <c r="O2">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>4</v>
       </c>
-      <c r="P2" s="5"/>
+      <c r="P2" s="4"/>
       <c r="Q2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="B3" s="16"/>
+      <c r="A3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="15"/>
       <c r="C3" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
       </c>
-      <c r="D3" s="5"/>
+      <c r="D3" s="4"/>
       <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="str">
+      <c r="F3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="G3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="H3" s="16"/>
+      <c r="G3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="H3" s="15"/>
       <c r="I3" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
-      <c r="J3" s="5"/>
+      <c r="J3" s="4"/>
       <c r="K3" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="9" t="str">
+      <c r="L3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="M3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="N3" s="16"/>
+      <c r="M3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="N3" s="15"/>
       <c r="O3" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Low</v>
       </c>
-      <c r="P3" s="5"/>
+      <c r="P3" s="4"/>
       <c r="Q3" t="s">
         <v>5</v>
       </c>
@@ -3275,76 +3209,76 @@
       </c>
     </row>
     <row r="4" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="16" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16" t="s">
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
     </row>
     <row r="5" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
     </row>
     <row r="6" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="16" t="s">
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16" t="s">
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
     </row>
     <row r="7" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -3362,7 +3296,7 @@
       <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="11" t="s">
         <v>2</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -3380,7 +3314,7 @@
       <c r="K7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="11" t="s">
         <v>2</v>
       </c>
       <c r="M7" s="1" t="s">
@@ -3403,207 +3337,207 @@
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A8" s="5">
+      <c r="A8" s="4">
         <v>1</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="B8" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" s="4">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="M8" s="4">
+        <v>1</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G9" s="4">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="M9" s="4">
+        <v>2</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="4">
+        <v>3</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="M10" s="4">
+        <v>3</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>4</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G11" s="4">
+        <v>4</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J11" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G8" s="5">
-        <v>1</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="M8" s="5">
-        <v>1</v>
-      </c>
-      <c r="N8" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
-        <v>2</v>
-      </c>
-      <c r="B9" s="4" t="s">
+      <c r="M11" s="4">
+        <v>4</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="M12" s="4">
+        <v>5</v>
+      </c>
+      <c r="N12" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="O12" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="G9" s="5">
-        <v>2</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="M9" s="5">
-        <v>2</v>
-      </c>
-      <c r="N9" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="P9" s="4" t="s">
+      <c r="P12" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>6</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="M13" s="4">
+        <v>6</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="O13" s="3" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="5">
-        <v>3</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="G10" s="5">
-        <v>3</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="M10" s="5">
-        <v>3</v>
-      </c>
-      <c r="N10" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="5">
-        <v>4</v>
-      </c>
-      <c r="B11" s="4" t="s">
+      <c r="P13" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="G11" s="5">
-        <v>4</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="M11" s="5">
-        <v>4</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="O11" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="5">
-        <v>5</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="M12" s="5">
-        <v>5</v>
-      </c>
-      <c r="N12" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="O12" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="P12" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="5">
-        <v>6</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="M13" s="5">
-        <v>6</v>
-      </c>
-      <c r="N13" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="O13" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="P13" s="4" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -3611,27 +3545,27 @@
         <v>7</v>
       </c>
       <c r="N14" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="O14" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="P14" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="29" x14ac:dyDescent="0.35">
-      <c r="M15" s="5">
+      <c r="M15" s="4">
         <v>8</v>
       </c>
-      <c r="N15" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="O15" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="P15" s="4" t="s">
-        <v>147</v>
+      <c r="N15" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="P15" s="3" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
@@ -3639,41 +3573,41 @@
         <v>9</v>
       </c>
       <c r="N16" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="O16" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="P16" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17" spans="13:16" ht="29" x14ac:dyDescent="0.35">
       <c r="M17">
         <v>10</v>
       </c>
-      <c r="N17" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="P17" s="4" t="s">
-        <v>147</v>
+      <c r="N17" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="P17" s="3" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="13:16" x14ac:dyDescent="0.35">
-      <c r="M18" s="5">
+      <c r="M18" s="4">
         <v>11</v>
       </c>
       <c r="N18" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="O18" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="P18" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="13:16" x14ac:dyDescent="0.35">
@@ -3681,27 +3615,27 @@
         <v>12</v>
       </c>
       <c r="N19" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="O19" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="P19" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="13:16" x14ac:dyDescent="0.35">
-      <c r="M20" s="5">
+      <c r="M20" s="4">
         <v>13</v>
       </c>
       <c r="N20" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="O20" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="P20" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="13:16" x14ac:dyDescent="0.35">
@@ -3709,13 +3643,13 @@
         <v>14</v>
       </c>
       <c r="N21" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="O21" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="P21" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -3750,13 +3684,13 @@
     <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.453125" customWidth="1"/>
     <col min="9" max="9" width="27.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30.26953125" customWidth="1"/>
     <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" style="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="35.453125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.54296875" customWidth="1"/>
@@ -3766,59 +3700,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
+      <c r="A1" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="8">
+      <c r="B2" s="15"/>
+      <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>5</v>
       </c>
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="8">
+      <c r="H2" s="15"/>
+      <c r="I2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>6</v>
       </c>
       <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="M2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="14">
+      <c r="N2" s="15"/>
+      <c r="O2" s="13">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>7</v>
       </c>
@@ -3827,41 +3761,41 @@
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="8" t="str">
+      <c r="A3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="15"/>
+      <c r="C3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="str">
+      <c r="F3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="G3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="H3" s="16"/>
-      <c r="I3" s="8" t="str">
+      <c r="G3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="H3" s="15"/>
+      <c r="I3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
       <c r="K3" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="9" t="str">
+      <c r="L3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="M3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="N3" s="16"/>
-      <c r="O3" s="14" t="str">
+      <c r="M3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="N3" s="15"/>
+      <c r="O3" s="13" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Low</v>
       </c>
@@ -3874,76 +3808,76 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="18" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="16" t="s">
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="18" t="s">
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="16" t="s">
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -3961,7 +3895,7 @@
       <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="11" t="s">
         <v>2</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -3979,7 +3913,7 @@
       <c r="K7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="11" t="s">
         <v>2</v>
       </c>
       <c r="M7" s="1" t="s">
@@ -4002,105 +3936,105 @@
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A8" s="5">
+      <c r="A8" s="4">
         <v>1</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>73</v>
+      <c r="B8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
-      <c r="H8" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>76</v>
+      <c r="H8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>57</v>
       </c>
       <c r="M8">
         <v>1</v>
       </c>
-      <c r="N8" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="O8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>76</v>
+      <c r="N8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
+      <c r="A9" s="4">
         <v>2</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>39</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>30</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>79</v>
+      <c r="H9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="M9">
         <v>2</v>
       </c>
-      <c r="N9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>79</v>
+      <c r="N9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="29" x14ac:dyDescent="0.35">
       <c r="G10">
         <v>3</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>104</v>
+      <c r="H10" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>85</v>
       </c>
       <c r="M10">
         <v>3</v>
       </c>
-      <c r="N10" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>104</v>
+      <c r="N10" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
@@ -4108,25 +4042,25 @@
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="J11" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="M11">
         <v>4</v>
       </c>
       <c r="N11" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="O11" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="P11" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
@@ -4134,25 +4068,25 @@
         <v>5</v>
       </c>
       <c r="H12" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="I12" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="J12" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="M12">
         <v>5</v>
       </c>
       <c r="N12" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="O12" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="P12" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
@@ -4160,25 +4094,25 @@
         <v>6</v>
       </c>
       <c r="H13" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="I13" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="J13" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="M13">
         <v>6</v>
       </c>
       <c r="N13" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="O13" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="P13" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -4186,19 +4120,19 @@
         <v>7</v>
       </c>
       <c r="H14" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="M14">
         <v>8</v>
       </c>
       <c r="N14" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="O14" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="P14" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
@@ -4206,25 +4140,25 @@
         <v>8</v>
       </c>
       <c r="H15" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="J15" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="M15">
         <v>9</v>
       </c>
       <c r="N15" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="O15" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="P15" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
@@ -4232,25 +4166,25 @@
         <v>9</v>
       </c>
       <c r="H16" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="J16" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="M16">
         <v>10</v>
       </c>
       <c r="N16" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="O16" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="P16" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="7:10" x14ac:dyDescent="0.35">
@@ -4258,13 +4192,13 @@
         <v>10</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="I17" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="J17" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="7:10" x14ac:dyDescent="0.35">
@@ -4272,13 +4206,13 @@
         <v>11</v>
       </c>
       <c r="H18" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="I18" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="J18" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="7:10" x14ac:dyDescent="0.35">
@@ -4286,13 +4220,13 @@
         <v>12</v>
       </c>
       <c r="H19" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="I19" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="J19" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="7:10" x14ac:dyDescent="0.35">
@@ -4300,13 +4234,13 @@
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="I20" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="J20" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="7:10" x14ac:dyDescent="0.35">
@@ -4314,13 +4248,13 @@
         <v>14</v>
       </c>
       <c r="H21" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="I21" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="J21" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="7:10" x14ac:dyDescent="0.35">
@@ -4328,13 +4262,13 @@
         <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="I22" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="J22" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="7:10" x14ac:dyDescent="0.35">
@@ -4342,13 +4276,13 @@
         <v>16</v>
       </c>
       <c r="H23" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="I23" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="J23" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="7:10" x14ac:dyDescent="0.35">
@@ -4356,13 +4290,13 @@
         <v>17</v>
       </c>
       <c r="H24" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="I24" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="J24" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="7:10" x14ac:dyDescent="0.35">
@@ -4370,13 +4304,13 @@
         <v>18</v>
       </c>
       <c r="H25" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="I25" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="J25" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -4411,13 +4345,13 @@
     <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" style="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="28.54296875" customWidth="1"/>
     <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.1796875" style="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="22.453125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="22.81640625" bestFit="1" customWidth="1"/>
@@ -4427,59 +4361,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="8">
+      <c r="B2" s="15"/>
+      <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>8</v>
       </c>
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="8">
+      <c r="H2" s="15"/>
+      <c r="I2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>9</v>
       </c>
       <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="M2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="8">
+      <c r="N2" s="15"/>
+      <c r="O2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>10</v>
       </c>
@@ -4488,41 +4422,41 @@
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="8" t="str">
+      <c r="A3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="15"/>
+      <c r="C3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="str">
+      <c r="F3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="G3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="H3" s="16"/>
-      <c r="I3" s="8" t="str">
+      <c r="G3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="H3" s="15"/>
+      <c r="I3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
       <c r="K3" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="9" t="str">
+      <c r="L3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="M3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="N3" s="16"/>
-      <c r="O3" s="8" t="str">
+      <c r="M3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="N3" s="15"/>
+      <c r="O3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Low</v>
       </c>
@@ -4535,76 +4469,76 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A4" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="19" t="s">
+      <c r="A4" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="20" t="s">
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="20"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="20"/>
-      <c r="R5" s="20"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A6" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="18" t="s">
+      <c r="A6" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="16" t="s">
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -4622,7 +4556,7 @@
       <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="11" t="s">
         <v>2</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -4640,7 +4574,7 @@
       <c r="K7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="11" t="s">
         <v>2</v>
       </c>
       <c r="M7" s="1" t="s">
@@ -4662,126 +4596,126 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="4">
+    <row r="8" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
         <v>1</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="4">
+      <c r="B8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="14"/>
+      <c r="G8" s="3">
         <v>1</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="L8" s="15"/>
-      <c r="M8" s="4">
+      <c r="H8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L8" s="14"/>
+      <c r="M8" s="3">
         <v>1</v>
       </c>
-      <c r="N8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" s="4" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
+      <c r="N8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="14"/>
+      <c r="G9" s="3">
+        <v>2</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="4">
+      <c r="I9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9" s="14"/>
+      <c r="M9" s="3">
         <v>2</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="L9" s="15"/>
-      <c r="M9" s="4">
-        <v>2</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="F10" s="15"/>
-      <c r="G10" s="4">
+      <c r="N9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="F10" s="14"/>
+      <c r="G10" s="3">
         <v>3</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="L10" s="15"/>
-      <c r="M10" s="4">
+      <c r="H10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L10" s="14"/>
+      <c r="M10" s="3">
         <v>3</v>
       </c>
-      <c r="N10" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>82</v>
+      <c r="N10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="29" x14ac:dyDescent="0.35">
-      <c r="M11" s="4">
+      <c r="M11" s="3">
         <v>4</v>
       </c>
-      <c r="N11" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="O11" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>85</v>
+      <c r="N11" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4808,333 +4742,212 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4413619-C528-4B04-A1ED-B4C77CA83066}">
-  <dimension ref="A1:AD12"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7265625" style="9"/>
+    <col min="6" max="6" width="8.7265625" style="8"/>
     <col min="7" max="7" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="48.81640625" customWidth="1"/>
-    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.453125" customWidth="1"/>
-    <col min="12" max="12" width="8.7265625" style="9"/>
-    <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30.81640625" customWidth="1"/>
-    <col min="16" max="16" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.7265625" style="9"/>
-    <col min="19" max="19" width="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.26953125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="41" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.7265625" style="9"/>
-    <col min="25" max="25" width="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.36328125" customWidth="1"/>
+    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.7265625" style="23"/>
+    <col min="14" max="14" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="41" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="17"/>
-      <c r="S1" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="T1" s="16"/>
-      <c r="U1" s="16"/>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="X1" s="17"/>
-      <c r="Y1" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="Z1" s="16"/>
-      <c r="AA1" s="16"/>
-      <c r="AB1" s="16"/>
-      <c r="AC1" s="16"/>
-      <c r="AD1" s="16"/>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="16"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2">
+      <c r="B2" s="15"/>
+      <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>11</v>
       </c>
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="8">
+      <c r="H2" s="15"/>
+      <c r="I2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>12</v>
       </c>
       <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="M2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="8">
+      <c r="N2" s="24"/>
+      <c r="O2" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>13</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="S2" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="T2" s="16"/>
-      <c r="U2" s="8">
-        <f>IFERROR(_xlfn.XLOOKUP(S1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
-        <v>14</v>
-      </c>
-      <c r="W2" t="s">
-        <v>4</v>
-      </c>
-      <c r="Y2" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z2" s="16"/>
-      <c r="AA2" s="8">
-        <f>IFERROR(_xlfn.XLOOKUP(Y1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
-        <v>15</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" t="str">
+      <c r="R2" s="8"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="15"/>
+      <c r="C3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="str">
+      <c r="F3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
       </c>
-      <c r="G3" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="H3" s="16"/>
-      <c r="I3" s="8" t="str">
+      <c r="G3" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="H3" s="15"/>
+      <c r="I3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
       </c>
       <c r="K3" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="9" t="str">
+      <c r="L3" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
       </c>
-      <c r="M3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="N3" s="16"/>
-      <c r="O3" s="8" t="str">
+      <c r="M3" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="N3" s="24"/>
+      <c r="O3" s="25" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="R3" s="9" t="str">
+      <c r="R3" s="8" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
-      <c r="S3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="T3" s="16"/>
-      <c r="U3" s="8" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(S1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
-        <v>Low</v>
-      </c>
-      <c r="W3" t="s">
-        <v>5</v>
-      </c>
-      <c r="X3" s="9" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(S1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
-        <v>Low</v>
-      </c>
-      <c r="Y3" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="8" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(Y1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
-        <v>High</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>5</v>
-      </c>
-      <c r="AD3" t="str">
-        <f>IFERROR(_xlfn.XLOOKUP(Y1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
-        <v>High</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="21"/>
-      <c r="S4" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20"/>
-      <c r="W4" s="20"/>
-      <c r="X4" s="21"/>
-      <c r="Y4" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z4" s="20"/>
-      <c r="AA4" s="20"/>
-      <c r="AB4" s="20"/>
-      <c r="AC4" s="20"/>
-      <c r="AD4" s="20"/>
-    </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="20"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="20"/>
-      <c r="T5" s="20"/>
-      <c r="U5" s="20"/>
-      <c r="V5" s="20"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="21"/>
-      <c r="Y5" s="20"/>
-      <c r="Z5" s="20"/>
-      <c r="AA5" s="20"/>
-      <c r="AB5" s="20"/>
-      <c r="AC5" s="20"/>
-      <c r="AD5" s="20"/>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="A6" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="17"/>
-      <c r="S6" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="T6" s="16"/>
-      <c r="U6" s="16"/>
-      <c r="V6" s="16"/>
-      <c r="W6" s="16"/>
-      <c r="X6" s="17"/>
-      <c r="Y6" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="Z6" s="16"/>
-      <c r="AA6" s="16"/>
-      <c r="AB6" s="16"/>
-      <c r="AC6" s="16"/>
-      <c r="AD6" s="16"/>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:18" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="20"/>
+    </row>
+    <row r="5" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="20"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A6" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="16"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -5150,7 +4963,7 @@
       <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="11" t="s">
         <v>2</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -5168,10 +4981,10 @@
       <c r="K7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" s="22" t="s">
         <v>0</v>
       </c>
       <c r="N7" s="1" t="s">
@@ -5186,296 +4999,281 @@
       <c r="Q7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="R7" s="12" t="s">
+      <c r="R7" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="S7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="W7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="X7" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="Y7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="AB7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AC7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="AD7" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>181</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="I8" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="J8" t="s">
-        <v>35</v>
-      </c>
-      <c r="M8">
+        <v>48</v>
+      </c>
+      <c r="M8" s="23">
         <v>1</v>
       </c>
-      <c r="N8" t="s">
-        <v>40</v>
-      </c>
-      <c r="O8" t="s">
-        <v>26</v>
-      </c>
-      <c r="P8" t="s">
-        <v>41</v>
-      </c>
-      <c r="S8">
-        <v>1</v>
-      </c>
-      <c r="T8" t="s">
-        <v>51</v>
-      </c>
-      <c r="U8" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y8">
-        <v>1</v>
-      </c>
-      <c r="Z8" t="s">
-        <v>62</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" ht="58" x14ac:dyDescent="0.35">
+      <c r="R8" s="8"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>182</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
       <c r="H9" t="s">
-        <v>34</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="M9">
+        <v>171</v>
+      </c>
+      <c r="I9" t="s">
+        <v>172</v>
+      </c>
+      <c r="J9" t="s">
+        <v>173</v>
+      </c>
+      <c r="M9" s="23">
         <v>2</v>
       </c>
-      <c r="N9" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="S9">
-        <v>2</v>
-      </c>
-      <c r="T9" t="s">
-        <v>55</v>
-      </c>
-      <c r="U9" t="s">
-        <v>57</v>
-      </c>
-      <c r="Y9">
-        <v>2</v>
-      </c>
-      <c r="Z9" t="s">
-        <v>191</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>192</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="R9" s="8"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>183</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="G10">
         <v>3</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>174</v>
       </c>
       <c r="I10" t="s">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="J10" t="s">
-        <v>59</v>
-      </c>
-      <c r="M10">
+        <v>176</v>
+      </c>
+      <c r="M10" s="23">
         <v>3</v>
       </c>
-      <c r="N10" t="s">
-        <v>45</v>
-      </c>
-      <c r="O10" t="s">
-        <v>46</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="S10">
-        <v>3</v>
-      </c>
-      <c r="T10" t="s">
-        <v>54</v>
-      </c>
-      <c r="U10" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y10">
-        <v>3</v>
-      </c>
-      <c r="Z10" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="R10" s="8"/>
+    </row>
+    <row r="11" spans="1:18" ht="58" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>4</v>
       </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" t="s">
-        <v>37</v>
-      </c>
-      <c r="S11">
+      <c r="B11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11">
         <v>4</v>
       </c>
-      <c r="T11" t="s">
-        <v>51</v>
-      </c>
-      <c r="U11" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="H11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" t="s">
+        <v>47</v>
+      </c>
+      <c r="M11" s="23">
+        <v>4</v>
+      </c>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="R11" s="8"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
-      </c>
-      <c r="S12">
-        <v>5</v>
-      </c>
-      <c r="T12" t="s">
-        <v>53</v>
-      </c>
-      <c r="U12" t="s">
-        <v>57</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>179</v>
+      </c>
+      <c r="D14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="15">
     <mergeCell ref="M1:R1"/>
-    <mergeCell ref="G4:L5"/>
-    <mergeCell ref="G6:L6"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="M3:N3"/>
     <mergeCell ref="M4:R5"/>
     <mergeCell ref="M6:R6"/>
     <mergeCell ref="G1:L1"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="G4:L5"/>
+    <mergeCell ref="G6:L6"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="Y1:AD1"/>
-    <mergeCell ref="Y2:Z2"/>
-    <mergeCell ref="Y3:Z3"/>
-    <mergeCell ref="S4:X5"/>
-    <mergeCell ref="S6:X6"/>
-    <mergeCell ref="Y4:AD5"/>
-    <mergeCell ref="Y6:AD6"/>
-    <mergeCell ref="S2:T2"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="S1:X1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Finish FileManagementTesting GUI test
</commit_message>
<xml_diff>
--- a/Test Cases.xlsx
+++ b/Test Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endresshauser-my.sharepoint.com/personal/corbin_ferguson_endress_com/Documents/Thesis Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1699" documentId="11_AD4DB114E441178AC67DF4D41ED1D894683EDF27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F63269EF-56D4-480B-B9BE-A1F71BFA4520}"/>
+  <xr:revisionPtr revIDLastSave="1708" documentId="11_AD4DB114E441178AC67DF4D41ED1D894683EDF27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6CF5F09-A140-4CE7-B7DC-37D3CDB6428F}"/>
   <bookViews>
     <workbookView xWindow="53880" yWindow="-5145" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="187">
   <si>
     <t>Step</t>
   </si>
@@ -170,9 +170,6 @@
     <t>File to load selected</t>
   </si>
   <si>
-    <t>doc object in Execute.cs updated to new object</t>
-  </si>
-  <si>
     <t>Confirm File Creation</t>
   </si>
   <si>
@@ -182,9 +179,6 @@
     <t>Preconditions: Empty template file loaded into application</t>
   </si>
   <si>
-    <t>Load File with error</t>
-  </si>
-  <si>
     <t>"Ok" button pressed</t>
   </si>
   <si>
@@ -195,9 +189,6 @@
   </si>
   <si>
     <t>New file created at location, return to action select window</t>
-  </si>
-  <si>
-    <t>File successfully loaded</t>
   </si>
   <si>
     <t>Error window appears with errors displayed</t>
@@ -832,6 +823,15 @@
   </si>
   <si>
     <t>ActionSelectLosecontrol</t>
+  </si>
+  <si>
+    <t>File successfully loaded, return to actionSelect</t>
+  </si>
+  <si>
+    <t>SaveFileButton</t>
+  </si>
+  <si>
+    <t>NewFileButton</t>
   </si>
 </sst>
 </file>
@@ -907,7 +907,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -941,6 +941,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -950,26 +952,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1934,6 +1923,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Corbin Ferguson" refreshedDate="46035.626586689817" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="17" xr:uid="{32ED145B-7CBC-4C3A-9787-F34239E1DCF7}">
   <cacheSource type="worksheet">
@@ -2374,29 +2367,29 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" t="s">
         <v>139</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" t="s">
-        <v>142</v>
-      </c>
       <c r="E1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G1">
         <f>COUNTIF(TestMaster[Test Status], "Not Implemented")</f>
         <v>13</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -2409,20 +2402,20 @@
         <v>Import Select Redundant Name</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G2">
         <f>COUNTIF(TestMaster[Test Status], "Pass")</f>
         <v>0</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I2">
         <v>17</v>
@@ -2438,20 +2431,20 @@
         <v>Element Quantity Creation</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" t="s">
         <v>144</v>
-      </c>
-      <c r="D3" t="s">
-        <v>145</v>
-      </c>
-      <c r="E3" t="s">
-        <v>147</v>
       </c>
       <c r="G3">
         <f>COUNTIF(TestMaster[Test Status], "Fail")</f>
         <v>0</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="I3">
         <v>17</v>
@@ -2467,10 +2460,10 @@
         <v>Nameless Module Creation</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G4">
         <f>COUNTIF(TestMaster[Test Status], "Not Run")</f>
@@ -2487,10 +2480,10 @@
         <v>Redundant Element Creation</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E5" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -2503,10 +2496,10 @@
         <v>No Element to Modify</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -2519,10 +2512,10 @@
         <v>Completed Element Modification</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E7" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -2535,10 +2528,10 @@
         <v>Modify into Redundant Element Name</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E8" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -2551,10 +2544,10 @@
         <v>Delete No Element Type</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -2567,10 +2560,10 @@
         <v>Delete Element Found</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E10" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
@@ -2583,10 +2576,10 @@
         <v>Delete Module by Port</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E11" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -2599,10 +2592,10 @@
         <v>FileManagementTesting</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E12" t="s">
         <v>144</v>
-      </c>
-      <c r="E12" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -2615,26 +2608,26 @@
         <v>ActionSelectLayout</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E13" t="s">
         <v>144</v>
       </c>
-      <c r="E13" t="s">
-        <v>147</v>
-      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="21">
+      <c r="A14">
         <f>ROW()-1</f>
         <v>13</v>
       </c>
-      <c r="B14" s="21" t="str">
+      <c r="B14" t="str">
         <f>'File Manipulation Testing'!M1</f>
         <v>ActionSelectLosecontrol</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E14" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2698,20 +2691,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="17"/>
       <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>1</v>
@@ -2721,10 +2714,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3" s="15"/>
+      <c r="A3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="17"/>
       <c r="C3" s="9" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
@@ -2738,32 +2731,32 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="16"/>
+      <c r="A4" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="18"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="16"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="18"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="18"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -2790,13 +2783,13 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C8" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
@@ -2805,13 +2798,13 @@
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -2820,13 +2813,13 @@
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -2835,13 +2828,13 @@
         <v>4</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
@@ -2850,13 +2843,13 @@
         <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
@@ -2865,13 +2858,13 @@
         <v>6</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
@@ -2880,13 +2873,13 @@
         <v>7</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="29" x14ac:dyDescent="0.35">
@@ -2895,13 +2888,13 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
@@ -2910,13 +2903,13 @@
         <v>9</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
@@ -2925,13 +2918,13 @@
         <v>10</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -2940,13 +2933,13 @@
         <v>11</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -2955,13 +2948,13 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -2970,13 +2963,13 @@
         <v>13</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -2985,13 +2978,13 @@
         <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C21" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
@@ -3000,13 +2993,13 @@
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -3015,13 +3008,13 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C23" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
@@ -3030,13 +3023,13 @@
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
@@ -3045,10 +3038,10 @@
         <v>18</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>30</v>
@@ -3093,36 +3086,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="15" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
     </row>
     <row r="2" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="17"/>
       <c r="C2">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>2</v>
@@ -3132,10 +3125,10 @@
         <v>4</v>
       </c>
       <c r="F2" s="8"/>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="15"/>
+      <c r="H2" s="17"/>
       <c r="I2">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>3</v>
@@ -3145,10 +3138,10 @@
         <v>4</v>
       </c>
       <c r="L2" s="8"/>
-      <c r="M2" s="15" t="s">
+      <c r="M2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="15"/>
+      <c r="N2" s="17"/>
       <c r="O2">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>4</v>
@@ -3159,10 +3152,10 @@
       </c>
     </row>
     <row r="3" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3" s="15"/>
+      <c r="A3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="17"/>
       <c r="C3" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
@@ -3175,10 +3168,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="H3" s="15"/>
+      <c r="G3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="H3" s="17"/>
       <c r="I3" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
@@ -3191,10 +3184,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="M3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="N3" s="15"/>
+      <c r="M3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="N3" s="17"/>
       <c r="O3" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Low</v>
@@ -3209,76 +3202,76 @@
       </c>
     </row>
     <row r="4" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="15" t="s">
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15" t="s">
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="15"/>
+      <c r="N4" s="17"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
     </row>
     <row r="5" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="17"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
+      <c r="R5" s="17"/>
     </row>
     <row r="6" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="15" t="s">
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15" t="s">
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
     </row>
     <row r="7" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -3341,37 +3334,37 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G8" s="4">
         <v>1</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="M8" s="4">
         <v>1</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -3379,37 +3372,37 @@
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G9" s="4">
         <v>2</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="M9" s="4">
         <v>2</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -3417,37 +3410,37 @@
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G10" s="4">
         <v>3</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="M10" s="4">
         <v>3</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -3455,37 +3448,37 @@
         <v>4</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G11" s="4">
         <v>4</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="M11" s="4">
         <v>4</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -3493,25 +3486,25 @@
         <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>116</v>
       </c>
       <c r="M12" s="4">
         <v>5</v>
       </c>
       <c r="N12" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="P12" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -3519,25 +3512,25 @@
         <v>6</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="M13" s="4">
         <v>6</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="O13" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="P13" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -3545,13 +3538,13 @@
         <v>7</v>
       </c>
       <c r="N14" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="P14" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -3559,13 +3552,13 @@
         <v>8</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="O15" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="P15" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
@@ -3573,13 +3566,13 @@
         <v>9</v>
       </c>
       <c r="N16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O16" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="P16" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="13:16" ht="29" x14ac:dyDescent="0.35">
@@ -3587,13 +3580,13 @@
         <v>10</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="O17" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="P17" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="P17" s="3" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="18" spans="13:16" x14ac:dyDescent="0.35">
@@ -3601,13 +3594,13 @@
         <v>11</v>
       </c>
       <c r="N18" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O18" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P18" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="13:16" x14ac:dyDescent="0.35">
@@ -3615,13 +3608,13 @@
         <v>12</v>
       </c>
       <c r="N19" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="O19" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="P19" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="13:16" x14ac:dyDescent="0.35">
@@ -3629,13 +3622,13 @@
         <v>13</v>
       </c>
       <c r="N20" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O20" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="P20" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="13:16" x14ac:dyDescent="0.35">
@@ -3643,22 +3636,17 @@
         <v>14</v>
       </c>
       <c r="N21" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="O21" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="P21" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="M1:R1"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="M3:N3"/>
@@ -3669,6 +3657,11 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G1:L1"/>
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A2:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3700,36 +3693,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="17" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="17"/>
       <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>5</v>
@@ -3737,10 +3730,10 @@
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="15"/>
+      <c r="H2" s="17"/>
       <c r="I2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>6</v>
@@ -3748,10 +3741,10 @@
       <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="15" t="s">
+      <c r="M2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="15"/>
+      <c r="N2" s="17"/>
       <c r="O2" s="13">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>7</v>
@@ -3761,10 +3754,10 @@
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3" s="15"/>
+      <c r="A3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="17"/>
       <c r="C3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
@@ -3776,10 +3769,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="H3" s="15"/>
+      <c r="G3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="H3" s="17"/>
       <c r="I3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
@@ -3791,10 +3784,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="M3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="N3" s="15"/>
+      <c r="M3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="N3" s="17"/>
       <c r="O3" s="13" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Low</v>
@@ -3808,76 +3801,76 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="17" t="s">
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="15" t="s">
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="15"/>
+      <c r="N4" s="17"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="17"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
+      <c r="R5" s="17"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17" t="s">
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="15" t="s">
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -3940,37 +3933,37 @@
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>21</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="M8">
         <v>1</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="O8" s="4" t="s">
         <v>21</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
@@ -3978,7 +3971,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>21</v>
@@ -3990,25 +3983,25 @@
         <v>2</v>
       </c>
       <c r="H9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>58</v>
-      </c>
       <c r="J9" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="M9">
         <v>2</v>
       </c>
       <c r="N9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="O9" s="3" t="s">
-        <v>58</v>
-      </c>
       <c r="P9" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -4016,25 +4009,25 @@
         <v>3</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="M10">
         <v>3</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
@@ -4042,25 +4035,25 @@
         <v>4</v>
       </c>
       <c r="H11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" t="s">
         <v>69</v>
       </c>
-      <c r="I11" t="s">
-        <v>72</v>
-      </c>
       <c r="J11" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="M11">
         <v>4</v>
       </c>
       <c r="N11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="O11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="P11" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
@@ -4068,25 +4061,25 @@
         <v>5</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="M12">
         <v>5</v>
       </c>
       <c r="N12" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="O12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
@@ -4094,25 +4087,25 @@
         <v>6</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I13" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J13" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="M13">
         <v>6</v>
       </c>
       <c r="N13" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="P13" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -4120,19 +4113,19 @@
         <v>7</v>
       </c>
       <c r="H14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="M14">
         <v>8</v>
       </c>
       <c r="N14" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="O14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="P14" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
@@ -4140,25 +4133,25 @@
         <v>8</v>
       </c>
       <c r="H15" t="s">
+        <v>66</v>
+      </c>
+      <c r="I15" t="s">
         <v>69</v>
       </c>
-      <c r="I15" t="s">
-        <v>72</v>
-      </c>
       <c r="J15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="M15">
         <v>9</v>
       </c>
       <c r="N15" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="O15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="P15" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
@@ -4166,25 +4159,25 @@
         <v>9</v>
       </c>
       <c r="H16" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I16" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="M16">
         <v>10</v>
       </c>
       <c r="N16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O16" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="P16" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="7:10" x14ac:dyDescent="0.35">
@@ -4192,13 +4185,13 @@
         <v>10</v>
       </c>
       <c r="H17" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="7:10" x14ac:dyDescent="0.35">
@@ -4206,13 +4199,13 @@
         <v>11</v>
       </c>
       <c r="H18" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J18" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="7:10" x14ac:dyDescent="0.35">
@@ -4220,13 +4213,13 @@
         <v>12</v>
       </c>
       <c r="H19" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I19" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="J19" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="7:10" x14ac:dyDescent="0.35">
@@ -4234,13 +4227,13 @@
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="I20" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J20" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="7:10" x14ac:dyDescent="0.35">
@@ -4248,13 +4241,13 @@
         <v>14</v>
       </c>
       <c r="H21" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I21" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="J21" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="7:10" x14ac:dyDescent="0.35">
@@ -4262,13 +4255,13 @@
         <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I22" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J22" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="7:10" x14ac:dyDescent="0.35">
@@ -4276,13 +4269,13 @@
         <v>16</v>
       </c>
       <c r="H23" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I23" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="J23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="7:10" x14ac:dyDescent="0.35">
@@ -4290,13 +4283,13 @@
         <v>17</v>
       </c>
       <c r="H24" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I24" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J24" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="7:10" x14ac:dyDescent="0.35">
@@ -4304,10 +4297,10 @@
         <v>18</v>
       </c>
       <c r="H25" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I25" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J25" t="s">
         <v>30</v>
@@ -4315,11 +4308,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
     <mergeCell ref="M1:R1"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="M3:N3"/>
@@ -4330,6 +4318,11 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G1:L1"/>
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4361,36 +4354,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="17" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="15" t="s">
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
-      <c r="P1" s="15"/>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="15"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="17"/>
       <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>8</v>
@@ -4398,10 +4391,10 @@
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="15"/>
+      <c r="H2" s="17"/>
       <c r="I2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>9</v>
@@ -4409,10 +4402,10 @@
       <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="15" t="s">
+      <c r="M2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="15"/>
+      <c r="N2" s="17"/>
       <c r="O2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>10</v>
@@ -4422,10 +4415,10 @@
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3" s="15"/>
+      <c r="A3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="17"/>
       <c r="C3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
@@ -4437,10 +4430,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="H3" s="15"/>
+      <c r="G3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="H3" s="17"/>
       <c r="I3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
@@ -4452,10 +4445,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Status], "Status not found"), "")</f>
         <v>Not Implemented</v>
       </c>
-      <c r="M3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="N3" s="15"/>
+      <c r="M3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="N3" s="17"/>
       <c r="O3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Low</v>
@@ -4469,76 +4462,76 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A4" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="18" t="s">
+      <c r="A4" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="19" t="s">
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A6" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17" t="s">
+      <c r="A6" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="15" t="s">
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -4601,39 +4594,39 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F8" s="14"/>
       <c r="G8" s="3">
         <v>1</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="L8" s="14"/>
       <c r="M8" s="3">
         <v>1</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>21</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:18" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -4641,7 +4634,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>21</v>
@@ -4654,26 +4647,26 @@
         <v>2</v>
       </c>
       <c r="H9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>58</v>
-      </c>
       <c r="J9" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L9" s="14"/>
       <c r="M9" s="3">
         <v>2</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:18" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -4682,26 +4675,26 @@
         <v>3</v>
       </c>
       <c r="H10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="J10" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="L10" s="14"/>
       <c r="M10" s="3">
         <v>3</v>
       </c>
       <c r="N10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O10" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="O10" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="P10" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="29" x14ac:dyDescent="0.35">
@@ -4709,22 +4702,17 @@
         <v>4</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A4:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
     <mergeCell ref="M1:R1"/>
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="M3:N3"/>
@@ -4735,6 +4723,11 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G1:L1"/>
+    <mergeCell ref="A4:F5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4756,7 +4749,7 @@
     <col min="9" max="9" width="27.36328125" customWidth="1"/>
     <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.7265625" style="23"/>
+    <col min="13" max="13" width="8.7265625" style="16"/>
     <col min="14" max="14" width="23.26953125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.1796875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="41" bestFit="1" customWidth="1"/>
@@ -4765,36 +4758,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="16"/>
+      <c r="A1" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="18"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="17"/>
       <c r="C2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>11</v>
@@ -4802,10 +4795,10 @@
       <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="15"/>
+      <c r="H2" s="17"/>
       <c r="I2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>12</v>
@@ -4813,25 +4806,24 @@
       <c r="K2" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="M2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="24"/>
-      <c r="O2" s="25">
+      <c r="N2" s="17"/>
+      <c r="O2" s="7">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test ID], "ID not found"), "")</f>
         <v>13</v>
       </c>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26" t="s">
+      <c r="Q2" t="s">
         <v>4</v>
       </c>
       <c r="R2" s="8"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3" s="15"/>
+      <c r="A3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="17"/>
       <c r="C3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
@@ -4843,10 +4835,10 @@
         <f>IFERROR(_xlfn.XLOOKUP(A1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="H3" s="15"/>
+      <c r="G3" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="H3" s="17"/>
       <c r="I3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
@@ -4858,16 +4850,15 @@
         <f>IFERROR(_xlfn.XLOOKUP(G1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>High</v>
       </c>
-      <c r="M3" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="N3" s="24"/>
-      <c r="O3" s="25" t="str">
+      <c r="M3" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="N3" s="17"/>
+      <c r="O3" s="7" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(M1, TestMaster[Test Name], TestMaster[Test Priority], "Priority not found"), "")</f>
         <v>Medium</v>
       </c>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="26" t="s">
+      <c r="Q3" t="s">
         <v>5</v>
       </c>
       <c r="R3" s="8" t="str">
@@ -4876,76 +4867,76 @@
       </c>
     </row>
     <row r="4" spans="1:18" s="2" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="19" t="s">
+      <c r="A4" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="18" t="s">
-        <v>185</v>
-      </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="21"/>
     </row>
     <row r="5" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="20"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="21"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A6" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="N6" s="24"/>
-      <c r="O6" s="24"/>
-      <c r="P6" s="24"/>
-      <c r="Q6" s="24"/>
-      <c r="R6" s="16"/>
+      <c r="A6" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="18"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -4984,7 +4975,7 @@
       <c r="L7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="M7" s="15" t="s">
         <v>0</v>
       </c>
       <c r="N7" s="1" t="s">
@@ -5008,27 +4999,27 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" t="s">
         <v>45</v>
       </c>
-      <c r="I8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J8" t="s">
-        <v>48</v>
-      </c>
-      <c r="M8" s="23">
+      <c r="M8" s="16">
         <v>1</v>
       </c>
       <c r="R8" s="8"/>
@@ -5038,27 +5029,27 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>179</v>
+      </c>
+      <c r="D9" t="s">
         <v>39</v>
-      </c>
-      <c r="C9" t="s">
-        <v>182</v>
-      </c>
-      <c r="D9" t="s">
-        <v>41</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
       <c r="H9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="I9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J9" t="s">
-        <v>173</v>
-      </c>
-      <c r="M9" s="23">
+        <v>170</v>
+      </c>
+      <c r="M9" s="16">
         <v>2</v>
       </c>
       <c r="R9" s="8"/>
@@ -5071,7 +5062,7 @@
         <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D10" t="s">
         <v>32</v>
@@ -5080,20 +5071,20 @@
         <v>3</v>
       </c>
       <c r="H10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="I10" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="J10" t="s">
-        <v>176</v>
-      </c>
-      <c r="M10" s="23">
+        <v>173</v>
+      </c>
+      <c r="M10" s="16">
         <v>3</v>
       </c>
       <c r="R10" s="8"/>
     </row>
-    <row r="11" spans="1:18" ht="58" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>4</v>
       </c>
@@ -5101,24 +5092,24 @@
         <v>33</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D11" t="s">
         <v>184</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="G11">
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I11" t="s">
         <v>21</v>
       </c>
       <c r="J11" t="s">
-        <v>47</v>
-      </c>
-      <c r="M11" s="23">
+        <v>44</v>
+      </c>
+      <c r="M11" s="16">
         <v>4</v>
       </c>
       <c r="N11" s="2"/>
@@ -5131,10 +5122,10 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
@@ -5142,10 +5133,13 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>176</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -5153,10 +5147,10 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>179</v>
-      </c>
-      <c r="D14" t="s">
-        <v>41</v>
+        <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
@@ -5164,10 +5158,10 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D15" t="s">
         <v>29</v>
@@ -5195,7 +5189,7 @@
         <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>185</v>
       </c>
       <c r="D17" t="s">
         <v>26</v>
@@ -5212,7 +5206,7 @@
         <v>27</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -5234,7 +5228,7 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
         <v>22</v>
@@ -5259,11 +5253,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="M1:R1"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="M4:R5"/>
-    <mergeCell ref="M6:R6"/>
     <mergeCell ref="G1:L1"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="G3:H3"/>
@@ -5274,6 +5263,11 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="M1:R1"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="M4:R5"/>
+    <mergeCell ref="M6:R6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cleanup for helper classes
</commit_message>
<xml_diff>
--- a/Test Cases.xlsx
+++ b/Test Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endresshauser-my.sharepoint.com/personal/corbin_ferguson_endress_com/Documents/ThesisBuildTool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="325" documentId="8_{B89245B7-08D9-4A9D-8516-F6C9C7AFFDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96FEFAAE-FE66-441B-92CD-2D085DA1D9DF}"/>
+  <xr:revisionPtr revIDLastSave="326" documentId="8_{B89245B7-08D9-4A9D-8516-F6C9C7AFFDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F37B63AB-F228-42AF-AB56-3D48E2C602AF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tests" sheetId="1" r:id="rId1"/>
@@ -1188,9 +1188,6 @@
     <t>Element Clash from import</t>
   </si>
   <si>
-    <t>"Cancel" selected from dropdown</t>
-  </si>
-  <si>
     <t>clashing elements window appears</t>
   </si>
   <si>
@@ -1198,6 +1195,9 @@
   </si>
   <si>
     <t>"TemplateLadderAOI" selected from dropdown</t>
+  </si>
+  <si>
+    <t>"Replace" selected from dropdown</t>
   </si>
 </sst>
 </file>
@@ -4583,7 +4583,7 @@
         <v>336</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>335</v>
@@ -4613,10 +4613,10 @@
         <v>337</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -4628,7 +4628,7 @@
         <v>381</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>42</v>

</xml_diff>